<commit_message>
weapon model + skin applied properly
</commit_message>
<xml_diff>
--- a/Docs/timesheet.xlsx
+++ b/Docs/timesheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Libraries\Documents\School\Y2\Personal Portfolio\pp2\UnrealEngineBasics\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alex\Documents\School\Y2\Personal Portfolio\pp2\UnrealEngineBasics\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A048823F-650E-422C-A1A7-8A1E3A470128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3B873D8-50A6-46F8-9CCD-5F57B962E823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Date/LO</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>REMAINING DAYS ASSUMED</t>
+  </si>
+  <si>
+    <t>BASED ON LAST DAY</t>
   </si>
 </sst>
 </file>
@@ -493,19 +496,19 @@
       </c>
       <c r="C3" s="1">
         <f>SUM(C5:C100)</f>
-        <v>19.383333333333329</v>
+        <v>19.549999999999994</v>
       </c>
       <c r="D3" s="1">
         <f>SUM(D5:D100)</f>
-        <v>9.7666666666666675</v>
+        <v>9.8666666666666671</v>
       </c>
       <c r="E3" s="1">
         <f>SUM(E5:E100)</f>
-        <v>14.183333333333334</v>
+        <v>14.366666666666667</v>
       </c>
       <c r="F3" s="1">
         <f>SUM(B3:E3)</f>
-        <v>46.849999999999994</v>
+        <v>47.29999999999999</v>
       </c>
       <c r="G3" s="1">
         <f>(1/60)*(180+20+10+6)</f>
@@ -513,11 +516,11 @@
       </c>
       <c r="H3" s="1">
         <f>F3+G3</f>
-        <v>50.449999999999996</v>
+        <v>50.899999999999991</v>
       </c>
       <c r="I3" s="1">
         <f>80-H3</f>
-        <v>29.550000000000004</v>
+        <v>29.100000000000009</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -533,24 +536,24 @@
       </c>
       <c r="C4" s="2">
         <f t="shared" ref="C4:E4" si="1">(C3/C2)</f>
-        <v>0.64611111111111097</v>
+        <v>0.65166666666666651</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>0.97666666666666679</v>
+        <v>0.98666666666666669</v>
       </c>
       <c r="E4" s="2">
         <f t="shared" si="1"/>
-        <v>0.4727777777777778</v>
+        <v>0.47888888888888892</v>
       </c>
       <c r="F4" s="2">
         <f>(F3/F2)</f>
-        <v>0.58562499999999995</v>
+        <v>0.59124999999999983</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="2">
         <f>(H3/F2)</f>
-        <v>0.63062499999999999</v>
+        <v>0.63624999999999987</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>12</v>
@@ -586,7 +589,7 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1">
         <f>F3/(COUNTA(A5:A100))</f>
-        <v>1.4640624999999998</v>
+        <v>1.4781249999999997</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
@@ -649,7 +652,7 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1">
         <f>I3/I5</f>
-        <v>20.183564567769483</v>
+        <v>19.687103594080348</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
@@ -681,7 +684,9 @@
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
+      <c r="I8" s="3" t="s">
+        <v>14</v>
+      </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
@@ -712,7 +717,10 @@
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
+      <c r="I9" s="1">
+        <f>I3/F33</f>
+        <v>9.9771428571428604</v>
+      </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
@@ -1439,20 +1447,20 @@
         <v>0.21666666666666667</v>
       </c>
       <c r="C33" s="1">
-        <f>(1/60)*(21+8)</f>
-        <v>0.48333333333333334</v>
+        <f>(1/60)*(21+8+10)</f>
+        <v>0.65</v>
       </c>
       <c r="D33" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f>(1/60)*(6)</f>
+        <v>0.1</v>
       </c>
       <c r="E33" s="1">
-        <f>(1/60)*(9+13+21+21+21+21)</f>
-        <v>1.7666666666666666</v>
+        <f>(1/60)*(9+13+21+21+21+21+11)</f>
+        <v>1.95</v>
       </c>
       <c r="F33" s="1">
         <f t="shared" ref="F33" si="13">SUM(B33:E33)</f>
-        <v>2.4666666666666668</v>
+        <v>2.9166666666666665</v>
       </c>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
@@ -1470,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="C34" s="1">
-        <f t="shared" si="3"/>
+        <f>(1/60)*(0)</f>
         <v>0</v>
       </c>
       <c r="D34" s="1">

</xml_diff>

<commit_message>
retargeted animations + guns can be changed
</commit_message>
<xml_diff>
--- a/Docs/timesheet.xlsx
+++ b/Docs/timesheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alex\Documents\School\Y2\Personal Portfolio\pp2\UnrealEngineBasics\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3B873D8-50A6-46F8-9CCD-5F57B962E823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18BECDE-0501-4553-A73E-C36255000668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,10 +77,10 @@
     <t>AVREAGE HR/DAY</t>
   </si>
   <si>
-    <t>REMAINING DAYS ASSUMED</t>
+    <t>BASED ON LAST DAY</t>
   </si>
   <si>
-    <t>BASED ON LAST DAY</t>
+    <t>REMAINING DAYS ASSUMED (AVERAGE)</t>
   </si>
 </sst>
 </file>
@@ -500,15 +500,15 @@
       </c>
       <c r="D3" s="1">
         <f>SUM(D5:D100)</f>
-        <v>9.8666666666666671</v>
+        <v>10.383333333333335</v>
       </c>
       <c r="E3" s="1">
         <f>SUM(E5:E100)</f>
-        <v>14.366666666666667</v>
+        <v>14.8</v>
       </c>
       <c r="F3" s="1">
         <f>SUM(B3:E3)</f>
-        <v>47.29999999999999</v>
+        <v>48.25</v>
       </c>
       <c r="G3" s="1">
         <f>(1/60)*(180+20+10+6)</f>
@@ -516,11 +516,11 @@
       </c>
       <c r="H3" s="1">
         <f>F3+G3</f>
-        <v>50.899999999999991</v>
+        <v>51.85</v>
       </c>
       <c r="I3" s="1">
-        <f>80-H3</f>
-        <v>29.100000000000009</v>
+        <f>80-F3</f>
+        <v>31.75</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -540,20 +540,20 @@
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>0.98666666666666669</v>
+        <v>1.0383333333333336</v>
       </c>
       <c r="E4" s="2">
         <f t="shared" si="1"/>
-        <v>0.47888888888888892</v>
+        <v>0.49333333333333335</v>
       </c>
       <c r="F4" s="2">
         <f>(F3/F2)</f>
-        <v>0.59124999999999983</v>
+        <v>0.60312500000000002</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="2">
         <f>(H3/F2)</f>
-        <v>0.63624999999999987</v>
+        <v>0.64812500000000006</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>12</v>
@@ -589,7 +589,7 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1">
         <f>F3/(COUNTA(A5:A100))</f>
-        <v>1.4781249999999997</v>
+        <v>1.5078125</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
@@ -620,7 +620,7 @@
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
       <c r="I6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
@@ -652,7 +652,7 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1">
         <f>I3/I5</f>
-        <v>19.687103594080348</v>
+        <v>21.05699481865285</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
@@ -685,7 +685,7 @@
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
@@ -719,7 +719,7 @@
       <c r="H9" s="1"/>
       <c r="I9" s="1">
         <f>I3/F33</f>
-        <v>9.9771428571428604</v>
+        <v>8.2112068965517242</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
@@ -1451,16 +1451,16 @@
         <v>0.65</v>
       </c>
       <c r="D33" s="1">
-        <f>(1/60)*(6)</f>
-        <v>0.1</v>
+        <f>(1/60)*(6+26+5)</f>
+        <v>0.6166666666666667</v>
       </c>
       <c r="E33" s="1">
-        <f>(1/60)*(9+13+21+21+21+21+11)</f>
-        <v>1.95</v>
+        <f>(1/60)*(9+13+21+21+21+21+11+26)</f>
+        <v>2.3833333333333333</v>
       </c>
       <c r="F33" s="1">
         <f t="shared" ref="F33" si="13">SUM(B33:E33)</f>
-        <v>2.9166666666666665</v>
+        <v>3.8666666666666667</v>
       </c>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>

</xml_diff>

<commit_message>
reload + ammo counter
</commit_message>
<xml_diff>
--- a/Docs/timesheet.xlsx
+++ b/Docs/timesheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alex\Documents\School\Y2\Personal Portfolio\pp2\UnrealEngineBasics\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Libraries\Documents\School\Y2\Personal Portfolio\pp2\UnrealEngineBasics\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18BECDE-0501-4553-A73E-C36255000668}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26CD587C-BC2C-43EC-87A4-70A73A8D4DBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -496,7 +496,7 @@
       </c>
       <c r="C3" s="1">
         <f>SUM(C5:C100)</f>
-        <v>19.549999999999994</v>
+        <v>19.666666666666661</v>
       </c>
       <c r="D3" s="1">
         <f>SUM(D5:D100)</f>
@@ -504,11 +504,11 @@
       </c>
       <c r="E3" s="1">
         <f>SUM(E5:E100)</f>
-        <v>14.8</v>
+        <v>15.666666666666668</v>
       </c>
       <c r="F3" s="1">
         <f>SUM(B3:E3)</f>
-        <v>48.25</v>
+        <v>49.233333333333334</v>
       </c>
       <c r="G3" s="1">
         <f>(1/60)*(180+20+10+6)</f>
@@ -516,11 +516,11 @@
       </c>
       <c r="H3" s="1">
         <f>F3+G3</f>
-        <v>51.85</v>
+        <v>52.833333333333336</v>
       </c>
       <c r="I3" s="1">
         <f>80-F3</f>
-        <v>31.75</v>
+        <v>30.766666666666666</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -536,7 +536,7 @@
       </c>
       <c r="C4" s="2">
         <f t="shared" ref="C4:E4" si="1">(C3/C2)</f>
-        <v>0.65166666666666651</v>
+        <v>0.65555555555555534</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
@@ -544,16 +544,16 @@
       </c>
       <c r="E4" s="2">
         <f t="shared" si="1"/>
-        <v>0.49333333333333335</v>
+        <v>0.52222222222222225</v>
       </c>
       <c r="F4" s="2">
         <f>(F3/F2)</f>
-        <v>0.60312500000000002</v>
+        <v>0.61541666666666672</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="2">
         <f>(H3/F2)</f>
-        <v>0.64812500000000006</v>
+        <v>0.66041666666666665</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>12</v>
@@ -589,7 +589,7 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1">
         <f>F3/(COUNTA(A5:A100))</f>
-        <v>1.5078125</v>
+        <v>1.5385416666666667</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
@@ -652,7 +652,7 @@
       <c r="H7" s="1"/>
       <c r="I7" s="1">
         <f>I3/I5</f>
-        <v>21.05699481865285</v>
+        <v>19.997291807718348</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
@@ -718,8 +718,8 @@
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1">
-        <f>I3/F33</f>
-        <v>8.2112068965517242</v>
+        <f>I3/F34</f>
+        <v>27.969696969696965</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
@@ -1474,24 +1474,24 @@
         <v>45335</v>
       </c>
       <c r="B34" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f>(1/60)*(7)</f>
+        <v>0.11666666666666667</v>
       </c>
       <c r="C34" s="1">
-        <f>(1/60)*(0)</f>
-        <v>0</v>
+        <f>(1/60)*(7)</f>
+        <v>0.11666666666666667</v>
       </c>
       <c r="D34" s="1">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="E34" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
+        <f>(1/60)*(22+22+8)</f>
+        <v>0.8666666666666667</v>
       </c>
       <c r="F34" s="1">
         <f t="shared" ref="F34:F37" si="14">SUM(B34:E34)</f>
-        <v>0</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>

</xml_diff>

<commit_message>
CROUCHING AND AIM OFFSET!!!!!
</commit_message>
<xml_diff>
--- a/Docs/timesheet.xlsx
+++ b/Docs/timesheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Libraries\Documents\School\Y2\Personal Portfolio\pp2\UnrealEngineBasics\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4916B2B4-24EF-4BC3-A952-CBAC7CB58BD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{174F99F8-96D5-43E8-B18D-CE9CFC11466E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Date/LO</t>
   </si>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>REMAINING DAYS ASSUMED (AVERAGE)</t>
+  </si>
+  <si>
+    <t>BASED ON TODAY</t>
   </si>
 </sst>
 </file>
@@ -496,11 +499,11 @@
       </c>
       <c r="C3" s="1">
         <f>SUM(C5:C100)</f>
-        <v>19.666666666666661</v>
+        <v>19.999999999999993</v>
       </c>
       <c r="D3" s="1">
         <f>SUM(D5:D100)</f>
-        <v>10.916666666666668</v>
+        <v>13.083333333333336</v>
       </c>
       <c r="E3" s="1">
         <f>SUM(E5:E100)</f>
@@ -508,7 +511,7 @@
       </c>
       <c r="F3" s="1">
         <f>SUM(B3:E3)</f>
-        <v>49.766666666666666</v>
+        <v>52.266666666666666</v>
       </c>
       <c r="G3" s="1">
         <f>(1/60)*(180+20+10+6)</f>
@@ -516,11 +519,11 @@
       </c>
       <c r="H3" s="1">
         <f>F3+G3</f>
-        <v>53.366666666666667</v>
+        <v>55.866666666666667</v>
       </c>
       <c r="I3" s="1">
         <f>80-F3</f>
-        <v>30.233333333333334</v>
+        <v>27.733333333333334</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -536,11 +539,11 @@
       </c>
       <c r="C4" s="2">
         <f t="shared" ref="C4:E4" si="1">(C3/C2)</f>
-        <v>0.65555555555555534</v>
+        <v>0.66666666666666641</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
-        <v>1.0916666666666668</v>
+        <v>1.3083333333333336</v>
       </c>
       <c r="E4" s="2">
         <f t="shared" si="1"/>
@@ -548,12 +551,12 @@
       </c>
       <c r="F4" s="2">
         <f>(F3/F2)</f>
-        <v>0.62208333333333332</v>
+        <v>0.65333333333333332</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="2">
         <f>(H3/F2)</f>
-        <v>0.66708333333333336</v>
+        <v>0.69833333333333336</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>12</v>
@@ -589,7 +592,7 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1">
         <f>F3/(COUNTA(A5:A100))</f>
-        <v>1.5552083333333333</v>
+        <v>1.6333333333333333</v>
       </c>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
@@ -651,8 +654,8 @@
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1">
-        <f>I3/I5</f>
-        <v>19.440053583389151</v>
+        <f>ROUNDUP(I3/I5, 0)</f>
+        <v>17</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
@@ -685,7 +688,7 @@
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
@@ -718,8 +721,8 @@
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1">
-        <f>I3/F34</f>
-        <v>18.510204081632654</v>
+        <f>ROUNDUP(I3/F34, 0)</f>
+        <v>7</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
@@ -751,7 +754,9 @@
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
+      <c r="I10" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -782,7 +787,10 @@
       </c>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
+      <c r="I11" s="1">
+        <f>ROUNDUP(I3/F33, 0)</f>
+        <v>8</v>
+      </c>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
@@ -1478,12 +1486,12 @@
         <v>0.11666666666666667</v>
       </c>
       <c r="C34" s="1">
-        <f>(1/60)*(7)</f>
-        <v>0.11666666666666667</v>
+        <f>(1/60)*(7+20)</f>
+        <v>0.45</v>
       </c>
       <c r="D34" s="1">
-        <f>(1/60)*(22+10)</f>
-        <v>0.53333333333333333</v>
+        <f>(1/60)*(22+10+20+20+20+20+5+20+5+20)</f>
+        <v>2.7</v>
       </c>
       <c r="E34" s="1">
         <f>(1/60)*(22+22+8)</f>
@@ -1491,7 +1499,7 @@
       </c>
       <c r="F34" s="1">
         <f t="shared" ref="F34:F37" si="14">SUM(B34:E34)</f>
-        <v>1.6333333333333333</v>
+        <v>4.1333333333333329</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>

</xml_diff>